<commit_message>
Minor app changes (#161) (#139)
* Minor app changes (#161)

* Fix pregnancy bug (#162)

* Added logic for pregnancy age and resolved pregnancy bug for below 9

* Adding updated app_settings

* Changed logic for isAdult function

* Worked on indentation and changed let to const (#163)

* Worked on indentation and changed let to const

* Undo file formatting

* Added translation for task group (#164)

* Added space (#165)
</commit_message>
<xml_diff>
--- a/forms/app/chv_quality_monitoring.xlsx
+++ b/forms/app/chv_quality_monitoring.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20387"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20389"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\D-tree\config-dtree-newrepo\config-dtree\forms\app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7F9D7F8-55AA-4E1A-8F31-5BDC62017991}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24C4C512-2915-4EC5-A60D-D9D20473565C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6590" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="551" uniqueCount="340">
   <si>
     <t>type</t>
   </si>
@@ -660,10 +660,6 @@
     <t>r_chw_info</t>
   </si>
   <si>
-    <t>&lt;div style="text-align:center;"&gt;&lt;span&gt;**CHV name:** ${chw_name}&lt;/span&gt; 
-&lt;span&gt;**CHV ID:** ${chw_id}&lt;/span&gt;&lt;/div&gt;</t>
-  </si>
-  <si>
     <t>r_improvement_areas_title</t>
   </si>
   <si>
@@ -946,10 +942,6 @@
     <t>Taarifa za CHV &lt;i class="fa fa-user"&gt;&lt;/i&gt;</t>
   </si>
   <si>
-    <t>&lt;div style="text-align:center;"&gt;&lt;span&gt;**Jina la CHV:** ${chw_name}&lt;/span&gt; 
-&lt;span&gt;**CHV ID:** ${chw_id}&lt;/span&gt;&lt;/div&gt;</t>
-  </si>
-  <si>
     <t>Maeneo ya maboresho &lt;i class="fa fa-flag"&gt;&lt;/i&gt;</t>
   </si>
   <si>
@@ -1143,6 +1135,18 @@
   <si>
     <t xml:space="preserve">Je muhudumu wa afya wa kujitolea anauliza na kuchunguza jinsi mlezi anavyomkosoa mtoto? </t>
   </si>
+  <si>
+    <t>&lt;div style="text-align:center;"&gt;&lt;span&gt;**CHV name:** ${chw_name}&lt;/span&gt;&lt;/div&gt;</t>
+  </si>
+  <si>
+    <t>&lt;div style="text-align:center;"&gt;&lt;span&gt;**Jina la CHV:** ${chw_name}&lt;/span&gt;&lt;/div&gt;</t>
+  </si>
+  <si>
+    <t>${next_follow_up_date}!='' and ${next_follow_up_date} &gt; today()</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tafadhali chagua tarehe ya mbele </t>
+  </si>
 </sst>
 </file>
 
@@ -1151,7 +1155,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dmmyyyyhm"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1204,6 +1208,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1222,10 +1233,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1276,9 +1288,16 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-00002F000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -4217,13 +4236,13 @@
         <v>42</v>
       </c>
       <c r="B79" s="11" t="s">
+        <v>271</v>
+      </c>
+      <c r="C79" s="18" t="s">
         <v>272</v>
       </c>
-      <c r="C79" s="18" t="s">
-        <v>273</v>
-      </c>
       <c r="D79" s="18" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="E79" s="19"/>
       <c r="F79" s="19"/>
@@ -4253,13 +4272,13 @@
         <v>52</v>
       </c>
       <c r="B80" s="11" t="s">
+        <v>273</v>
+      </c>
+      <c r="C80" s="21" t="s">
         <v>274</v>
       </c>
-      <c r="C80" s="21" t="s">
-        <v>275</v>
-      </c>
       <c r="D80" s="4" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="E80" s="19" t="s">
         <v>56</v>
@@ -4291,13 +4310,13 @@
         <v>52</v>
       </c>
       <c r="B81" s="11" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C81" s="21" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="E81" s="19" t="s">
         <v>56</v>
@@ -4329,13 +4348,13 @@
         <v>52</v>
       </c>
       <c r="B82" s="11" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C82" s="21" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="D82" s="19" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="E82" s="19" t="s">
         <v>56</v>
@@ -4367,13 +4386,13 @@
         <v>52</v>
       </c>
       <c r="B83" s="11" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C83" s="21" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="D83" s="4" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="E83" s="19" t="s">
         <v>56</v>
@@ -4405,13 +4424,13 @@
         <v>135</v>
       </c>
       <c r="B84" s="11" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C84" s="21" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="E84" s="19"/>
       <c r="F84" s="18"/>
@@ -4441,13 +4460,13 @@
         <v>52</v>
       </c>
       <c r="B85" s="11" t="s">
+        <v>279</v>
+      </c>
+      <c r="C85" s="18" t="s">
         <v>280</v>
       </c>
-      <c r="C85" s="18" t="s">
-        <v>281</v>
-      </c>
       <c r="D85" s="22" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="E85" s="19" t="s">
         <v>56</v>
@@ -4479,13 +4498,13 @@
         <v>42</v>
       </c>
       <c r="B86" s="11" t="s">
+        <v>281</v>
+      </c>
+      <c r="C86" s="18" t="s">
         <v>282</v>
       </c>
-      <c r="C86" s="18" t="s">
-        <v>283</v>
-      </c>
       <c r="D86" s="23" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="E86" s="19"/>
       <c r="F86" s="19"/>
@@ -4515,13 +4534,13 @@
         <v>52</v>
       </c>
       <c r="B87" s="11" t="s">
+        <v>283</v>
+      </c>
+      <c r="C87" s="18" t="s">
         <v>284</v>
       </c>
-      <c r="C87" s="18" t="s">
-        <v>285</v>
-      </c>
       <c r="D87" s="22" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="E87" s="19"/>
       <c r="F87" s="19"/>
@@ -4551,13 +4570,13 @@
         <v>52</v>
       </c>
       <c r="B88" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="C88" s="18" t="s">
         <v>286</v>
       </c>
-      <c r="C88" s="18" t="s">
-        <v>287</v>
-      </c>
       <c r="D88" s="22" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="E88" s="19"/>
       <c r="F88" s="19"/>
@@ -4587,13 +4606,13 @@
         <v>52</v>
       </c>
       <c r="B89" s="11" t="s">
+        <v>287</v>
+      </c>
+      <c r="C89" s="18" t="s">
         <v>288</v>
       </c>
-      <c r="C89" s="18" t="s">
-        <v>289</v>
-      </c>
       <c r="D89" s="22" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="E89" s="19"/>
       <c r="F89" s="19"/>
@@ -4623,13 +4642,13 @@
         <v>52</v>
       </c>
       <c r="B90" s="11" t="s">
+        <v>289</v>
+      </c>
+      <c r="C90" s="18" t="s">
         <v>290</v>
       </c>
-      <c r="C90" s="18" t="s">
-        <v>291</v>
-      </c>
       <c r="D90" s="22" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="E90" s="19"/>
       <c r="F90" s="19"/>
@@ -4659,13 +4678,13 @@
         <v>52</v>
       </c>
       <c r="B91" s="11" t="s">
+        <v>291</v>
+      </c>
+      <c r="C91" s="18" t="s">
         <v>292</v>
       </c>
-      <c r="C91" s="18" t="s">
-        <v>293</v>
-      </c>
       <c r="D91" s="22" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="E91" s="19"/>
       <c r="F91" s="19"/>
@@ -4695,13 +4714,13 @@
         <v>42</v>
       </c>
       <c r="B92" s="11" t="s">
+        <v>293</v>
+      </c>
+      <c r="C92" s="18" t="s">
         <v>294</v>
       </c>
-      <c r="C92" s="18" t="s">
-        <v>295</v>
-      </c>
       <c r="D92" s="23" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="E92" s="19"/>
       <c r="F92" s="19"/>
@@ -4731,13 +4750,13 @@
         <v>52</v>
       </c>
       <c r="B93" s="11" t="s">
+        <v>295</v>
+      </c>
+      <c r="C93" s="18" t="s">
         <v>296</v>
       </c>
-      <c r="C93" s="18" t="s">
-        <v>297</v>
-      </c>
       <c r="D93" s="19" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="E93" s="19"/>
       <c r="F93" s="19"/>
@@ -4767,13 +4786,13 @@
         <v>52</v>
       </c>
       <c r="B94" s="11" t="s">
+        <v>297</v>
+      </c>
+      <c r="C94" s="21" t="s">
         <v>298</v>
       </c>
-      <c r="C94" s="21" t="s">
-        <v>299</v>
-      </c>
       <c r="D94" s="22" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="E94" s="19"/>
       <c r="F94" s="19"/>
@@ -4803,13 +4822,13 @@
         <v>52</v>
       </c>
       <c r="B95" s="11" t="s">
+        <v>299</v>
+      </c>
+      <c r="C95" s="18" t="s">
         <v>300</v>
       </c>
-      <c r="C95" s="18" t="s">
-        <v>301</v>
-      </c>
       <c r="D95" s="22" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="E95" s="19"/>
       <c r="F95" s="19"/>
@@ -5682,7 +5701,7 @@
       <c r="I120" s="6"/>
       <c r="J120" s="6"/>
       <c r="K120" s="5" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="L120" s="6"/>
       <c r="M120" s="6"/>
@@ -5705,7 +5724,7 @@
         <v>33</v>
       </c>
       <c r="B121" s="6" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C121" s="6" t="s">
         <v>201</v>
@@ -5720,7 +5739,7 @@
       <c r="I121" s="6"/>
       <c r="J121" s="6"/>
       <c r="K121" s="6" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="L121" s="6"/>
       <c r="M121" s="6"/>
@@ -5758,7 +5777,7 @@
       <c r="I122" s="8"/>
       <c r="J122" s="8"/>
       <c r="K122" s="7" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="L122" s="7"/>
       <c r="M122" s="8"/>
@@ -5817,7 +5836,7 @@
         <v>205</v>
       </c>
       <c r="D124" s="10" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="E124" s="10"/>
       <c r="F124" s="10"/>
@@ -5855,7 +5874,7 @@
         <v>208</v>
       </c>
       <c r="D125" s="13" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E125" s="10"/>
       <c r="F125" s="10"/>
@@ -5882,7 +5901,7 @@
       <c r="Y125" s="4"/>
       <c r="Z125" s="4"/>
     </row>
-    <row r="126" spans="1:26" ht="26" x14ac:dyDescent="0.6">
+    <row r="126" spans="1:26" ht="13" x14ac:dyDescent="0.6">
       <c r="A126" s="9" t="s">
         <v>42</v>
       </c>
@@ -5890,10 +5909,10 @@
         <v>210</v>
       </c>
       <c r="C126" s="9" t="s">
-        <v>211</v>
+        <v>336</v>
       </c>
       <c r="D126" s="13" t="s">
-        <v>306</v>
+        <v>337</v>
       </c>
       <c r="E126" s="10"/>
       <c r="F126" s="10"/>
@@ -5923,18 +5942,18 @@
         <v>42</v>
       </c>
       <c r="B127" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="C127" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="C127" s="3" t="s">
-        <v>213</v>
-      </c>
       <c r="D127" s="4" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="E127" s="4"/>
       <c r="F127" s="4"/>
       <c r="G127" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="H127" s="4"/>
       <c r="I127" s="4"/>
@@ -5961,13 +5980,13 @@
         <v>42</v>
       </c>
       <c r="B128" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="C128" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="C128" s="3" t="s">
-        <v>216</v>
-      </c>
       <c r="D128" s="4" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="E128" s="4"/>
       <c r="F128" s="4"/>
@@ -5997,18 +6016,18 @@
         <v>42</v>
       </c>
       <c r="B129" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="C129" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="C129" s="9" t="s">
-        <v>218</v>
-      </c>
       <c r="D129" s="13" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="E129" s="10"/>
       <c r="F129" s="10"/>
       <c r="G129" s="11" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="H129" s="10"/>
       <c r="I129" s="10"/>
@@ -6035,13 +6054,13 @@
         <v>52</v>
       </c>
       <c r="B130" s="12" t="s">
+        <v>218</v>
+      </c>
+      <c r="C130" s="13" t="s">
         <v>219</v>
       </c>
-      <c r="C130" s="13" t="s">
-        <v>220</v>
-      </c>
       <c r="D130" s="13" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="E130" s="11" t="s">
         <v>56</v>
@@ -6070,31 +6089,33 @@
     </row>
     <row r="131" spans="1:26" ht="26" x14ac:dyDescent="0.6">
       <c r="A131" s="12" t="s">
+        <v>220</v>
+      </c>
+      <c r="B131" s="12" t="s">
         <v>221</v>
       </c>
-      <c r="B131" s="12" t="s">
+      <c r="C131" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="C131" s="3" t="s">
-        <v>223</v>
-      </c>
       <c r="D131" s="4" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="E131" s="3" t="s">
         <v>56</v>
       </c>
       <c r="F131" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G131" s="4"/>
       <c r="H131" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="I131" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="I131" s="3" t="s">
-        <v>226</v>
+      <c r="J131" s="4" t="s">
+        <v>339</v>
       </c>
-      <c r="J131" s="4"/>
       <c r="K131" s="4"/>
       <c r="L131" s="4"/>
       <c r="M131" s="4"/>
@@ -6117,7 +6138,7 @@
         <v>33</v>
       </c>
       <c r="B132" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C132" s="3" t="s">
         <v>201</v>
@@ -6127,14 +6148,14 @@
       </c>
       <c r="E132" s="4"/>
       <c r="F132" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G132" s="4"/>
       <c r="H132" s="4"/>
       <c r="I132" s="4"/>
       <c r="J132" s="4"/>
       <c r="K132" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="L132" s="4"/>
       <c r="M132" s="4"/>
@@ -6152,22 +6173,22 @@
       <c r="Y132" s="4"/>
       <c r="Z132" s="4"/>
     </row>
-    <row r="133" spans="1:26" ht="26" x14ac:dyDescent="0.6">
+    <row r="133" spans="1:26" ht="52" x14ac:dyDescent="0.6">
       <c r="A133" s="3" t="s">
         <v>42</v>
       </c>
       <c r="B133" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="C133" s="3" t="s">
         <v>229</v>
       </c>
-      <c r="C133" s="3" t="s">
-        <v>230</v>
-      </c>
       <c r="D133" s="4" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="E133" s="4"/>
-      <c r="F133" s="3" t="s">
-        <v>224</v>
+      <c r="F133" s="24" t="s">
+        <v>338</v>
       </c>
       <c r="G133" s="4"/>
       <c r="H133" s="4"/>
@@ -6195,7 +6216,7 @@
         <v>33</v>
       </c>
       <c r="B134" s="9" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C134" s="9" t="s">
         <v>201</v>
@@ -6210,7 +6231,7 @@
       <c r="I134" s="10"/>
       <c r="J134" s="10"/>
       <c r="K134" s="13" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="L134" s="10"/>
       <c r="M134" s="10"/>
@@ -6228,21 +6249,23 @@
       <c r="Y134" s="10"/>
       <c r="Z134" s="10"/>
     </row>
-    <row r="135" spans="1:26" ht="13" x14ac:dyDescent="0.6">
+    <row r="135" spans="1:26" ht="52" x14ac:dyDescent="0.6">
       <c r="A135" s="9" t="s">
         <v>42</v>
       </c>
       <c r="B135" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="C135" s="13" t="s">
         <v>233</v>
       </c>
-      <c r="C135" s="13" t="s">
-        <v>234</v>
-      </c>
       <c r="D135" s="13" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="E135" s="10"/>
-      <c r="F135" s="10"/>
+      <c r="F135" s="25" t="s">
+        <v>338</v>
+      </c>
       <c r="G135" s="10"/>
       <c r="H135" s="10"/>
       <c r="I135" s="10"/>
@@ -30395,7 +30418,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A1" s="14" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B1" s="14" t="s">
         <v>1</v>
@@ -30431,142 +30454,142 @@
     </row>
     <row r="2" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A2" s="16" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B2" s="16" t="s">
         <v>56</v>
       </c>
       <c r="C2" s="16" t="s">
+        <v>236</v>
+      </c>
+      <c r="D2" s="16" t="s">
         <v>237</v>
       </c>
-      <c r="D2" s="16" t="s">
+    </row>
+    <row r="3" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A3" s="16" t="s">
+        <v>235</v>
+      </c>
+      <c r="B3" s="16" t="s">
         <v>238</v>
       </c>
-    </row>
-    <row r="3" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A3" s="16" t="s">
-        <v>236</v>
-      </c>
-      <c r="B3" s="16" t="s">
+      <c r="C3" s="16" t="s">
         <v>239</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="D3" s="16" t="s">
         <v>240</v>
       </c>
-      <c r="D3" s="16" t="s">
-        <v>241</v>
-      </c>
     </row>
     <row r="5" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A5" s="16" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B5" s="16" t="s">
         <v>56</v>
       </c>
       <c r="C5" s="16" t="s">
+        <v>236</v>
+      </c>
+      <c r="D5" s="16" t="s">
         <v>237</v>
       </c>
-      <c r="D5" s="16" t="s">
+    </row>
+    <row r="6" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A6" s="16" t="s">
+        <v>241</v>
+      </c>
+      <c r="B6" s="16" t="s">
         <v>238</v>
       </c>
-    </row>
-    <row r="6" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A6" s="16" t="s">
+      <c r="C6" s="16" t="s">
+        <v>239</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A7" s="16" t="s">
+        <v>241</v>
+      </c>
+      <c r="B7" s="16" t="s">
         <v>242</v>
       </c>
-      <c r="B6" s="16" t="s">
-        <v>239</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>240</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="7" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A7" s="16" t="s">
-        <v>242</v>
-      </c>
-      <c r="B7" s="16" t="s">
+      <c r="C7" s="16" t="s">
         <v>243</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="D7" s="16" t="s">
         <v>244</v>
       </c>
-      <c r="D7" s="16" t="s">
-        <v>245</v>
-      </c>
     </row>
     <row r="9" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A9" s="16" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B9" s="16">
         <v>0</v>
       </c>
       <c r="C9" s="16" t="s">
+        <v>246</v>
+      </c>
+      <c r="D9" s="16" t="s">
         <v>247</v>
       </c>
-      <c r="D9" s="16" t="s">
-        <v>248</v>
-      </c>
     </row>
     <row r="10" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A10" s="16" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B10" s="16">
         <v>1</v>
       </c>
       <c r="C10" s="16" t="s">
+        <v>248</v>
+      </c>
+      <c r="D10" s="16" t="s">
         <v>249</v>
       </c>
-      <c r="D10" s="16" t="s">
-        <v>250</v>
-      </c>
     </row>
     <row r="11" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A11" s="16" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B11" s="16">
         <v>2</v>
       </c>
       <c r="C11" s="16" t="s">
+        <v>250</v>
+      </c>
+      <c r="D11" s="16" t="s">
         <v>251</v>
       </c>
-      <c r="D11" s="16" t="s">
-        <v>252</v>
-      </c>
     </row>
     <row r="12" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A12" s="16" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B12" s="16">
         <v>3</v>
       </c>
       <c r="C12" s="16" t="s">
+        <v>252</v>
+      </c>
+      <c r="D12" s="16" t="s">
         <v>253</v>
       </c>
-      <c r="D12" s="16" t="s">
-        <v>254</v>
-      </c>
     </row>
     <row r="13" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A13" s="16" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B13" s="16">
         <v>5</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
@@ -30574,13 +30597,13 @@
         <v>171</v>
       </c>
       <c r="B15" s="16" t="s">
+        <v>256</v>
+      </c>
+      <c r="C15" s="16" t="s">
         <v>257</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="D15" s="16" t="s">
         <v>258</v>
-      </c>
-      <c r="D15" s="16" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
@@ -30588,13 +30611,13 @@
         <v>171</v>
       </c>
       <c r="B16" s="16" t="s">
+        <v>259</v>
+      </c>
+      <c r="C16" s="16" t="s">
         <v>260</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="D16" s="16" t="s">
         <v>261</v>
-      </c>
-      <c r="D16" s="16" t="s">
-        <v>262</v>
       </c>
     </row>
   </sheetData>
@@ -30615,22 +30638,22 @@
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>267</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>268</v>
       </c>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
@@ -30658,20 +30681,20 @@
         <v>161</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C2" s="17">
         <f ca="1">NOW()</f>
-        <v>44783.384753356484</v>
+        <v>44825.55971076389</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>269</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>270</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>271</v>
       </c>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>

</xml_diff>